<commit_message>
Update ecu_cofig BAS and display_name.json
</commit_message>
<xml_diff>
--- a/config/ecu_config.xlsx
+++ b/config/ecu_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\REDO\CODINGTOOL\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9566F2BA-2917-488B-BF93-441CEF1C8C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC4E8B6C-596C-4C44-9F21-E8335DFC2F47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ECU_list" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Animation dark mode button
</commit_message>
<xml_diff>
--- a/config/ecu_config.xlsx
+++ b/config/ecu_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\REDO\SW\EEIV Diagnostic_v1.0.0\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CB999EC-A825-4126-8240-B6AC58D4B199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D11CAB-13CE-44B2-8601-72665D217728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ECU_list" sheetId="1" r:id="rId1"/>
@@ -262,21 +262,12 @@
     <t>|VCU|</t>
   </si>
   <si>
-    <t>|2IN1|POD|PDU|DCDC1|DCCO_DCDC|</t>
-  </si>
-  <si>
     <t>|EDS|MCU|FMCU|EDS_F|</t>
   </si>
   <si>
     <t>|EAC|</t>
   </si>
   <si>
-    <t>|MHU|IVI|</t>
-  </si>
-  <si>
-    <t>|XGW|CVC|IVC|</t>
-  </si>
-  <si>
     <t>|AVAS|</t>
   </si>
   <si>
@@ -331,12 +322,6 @@
     <t>|USS_RR |EKS_1|</t>
   </si>
   <si>
-    <t>|DKCU|</t>
-  </si>
-  <si>
-    <t>|BPM|</t>
-  </si>
-  <si>
     <t>|DCDC_2|</t>
   </si>
   <si>
@@ -428,6 +413,21 @@
   </si>
   <si>
     <t>|BAS|</t>
+  </si>
+  <si>
+    <t>|BPM|BCM_BPM|</t>
+  </si>
+  <si>
+    <t>|2IN1|POD|PDU|DCDC1|DCCO_DCDC|3IN1|</t>
+  </si>
+  <si>
+    <t>|XGW|CVC|IVC|IVC_SGC</t>
+  </si>
+  <si>
+    <t>|MHU|IVI|IVC_MHU|</t>
+  </si>
+  <si>
+    <t>|VDKCU|</t>
   </si>
 </sst>
 </file>
@@ -892,7 +892,7 @@
     </row>
     <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>80</v>
+        <v>132</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>6</v>
@@ -903,7 +903,7 @@
     </row>
     <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>8</v>
@@ -914,7 +914,7 @@
     </row>
     <row r="10" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>10</v>
@@ -925,7 +925,7 @@
     </row>
     <row r="11" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>83</v>
+        <v>134</v>
       </c>
       <c r="B11" s="1">
         <v>684</v>
@@ -936,7 +936,7 @@
     </row>
     <row r="12" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>84</v>
+        <v>133</v>
       </c>
       <c r="B12" s="1">
         <v>682</v>
@@ -947,7 +947,7 @@
     </row>
     <row r="13" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>11</v>
@@ -958,7 +958,7 @@
     </row>
     <row r="14" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>13</v>
@@ -969,7 +969,7 @@
     </row>
     <row r="15" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>14</v>
@@ -980,7 +980,7 @@
     </row>
     <row r="16" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B16" s="1">
         <v>0</v>
@@ -991,7 +991,7 @@
     </row>
     <row r="17" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B17" s="1">
         <v>689</v>
@@ -1002,7 +1002,7 @@
     </row>
     <row r="18" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>17</v>
@@ -1013,7 +1013,7 @@
     </row>
     <row r="19" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B19" s="1">
         <v>686</v>
@@ -1024,7 +1024,7 @@
     </row>
     <row r="20" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>19</v>
@@ -1035,7 +1035,7 @@
     </row>
     <row r="21" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>21</v>
@@ -1046,7 +1046,7 @@
     </row>
     <row r="22" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>23</v>
@@ -1057,7 +1057,7 @@
     </row>
     <row r="23" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B23" s="1">
         <v>696</v>
@@ -1068,7 +1068,7 @@
     </row>
     <row r="24" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>25</v>
@@ -1079,7 +1079,7 @@
     </row>
     <row r="25" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>26</v>
@@ -1090,7 +1090,7 @@
     </row>
     <row r="26" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>27</v>
@@ -1101,7 +1101,7 @@
     </row>
     <row r="27" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>28</v>
@@ -1112,7 +1112,7 @@
     </row>
     <row r="28" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>29</v>
@@ -1123,7 +1123,7 @@
     </row>
     <row r="29" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>31</v>
@@ -1134,7 +1134,7 @@
     </row>
     <row r="30" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>32</v>
@@ -1145,7 +1145,7 @@
     </row>
     <row r="31" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>103</v>
+        <v>135</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>33</v>
@@ -1156,7 +1156,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>104</v>
+        <v>131</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>35</v>
@@ -1167,7 +1167,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>37</v>
@@ -1178,7 +1178,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>38</v>
@@ -1189,7 +1189,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B35" s="2">
         <v>683</v>
@@ -1200,7 +1200,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>40</v>
@@ -1211,7 +1211,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>41</v>
@@ -1222,7 +1222,7 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>42</v>
@@ -1233,7 +1233,7 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>44</v>
@@ -1244,7 +1244,7 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>46</v>
@@ -1255,7 +1255,7 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>47</v>
@@ -1266,7 +1266,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>48</v>
@@ -1277,7 +1277,7 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B43" s="2">
         <v>697</v>
@@ -1288,7 +1288,7 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>49</v>
@@ -1299,7 +1299,7 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>50</v>
@@ -1310,7 +1310,7 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>52</v>
@@ -1321,7 +1321,7 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>53</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>55</v>
@@ -1343,7 +1343,7 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>57</v>
@@ -1354,7 +1354,7 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>58</v>
@@ -1365,7 +1365,7 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B51" s="2">
         <v>685</v>
@@ -1376,7 +1376,7 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>59</v>
@@ -1387,7 +1387,7 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>61</v>
@@ -1398,7 +1398,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B54" s="2">
         <v>694</v>
@@ -1409,7 +1409,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>63</v>
@@ -1420,7 +1420,7 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B56" s="2">
         <v>695</v>
@@ -1431,7 +1431,7 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B57" s="2">
         <v>691</v>
@@ -1442,7 +1442,7 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>65</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>66</v>
@@ -1464,7 +1464,7 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>68</v>
@@ -1475,7 +1475,7 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>69</v>
@@ -1486,7 +1486,7 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>71</v>
@@ -1497,7 +1497,7 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>73</v>

</xml_diff>